<commit_message>
fix some of the metadata
</commit_message>
<xml_diff>
--- a/data/2026_06_30_RepoMetaCuration.xlsx
+++ b/data/2026_06_30_RepoMetaCuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gtsueng\Anaconda3\envs\nde\nde_meta_batch_converter\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4103D2DB-17C0-432B-AEC5-B638A7C9BAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D46906F-2EAD-40EB-92EF-108F65732A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12096" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="resource_base" sheetId="1" r:id="rId1"/>
@@ -46,12 +46,12 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={45597fe8-a5be-4e4c-93e8-ee11830187a8}</author>
-    <author>tc={5af53a1d-2122-4bf0-a09a-3fd230718d9d}</author>
-    <author>tc={e77d8335-66cc-4db9-adea-68353ee4d071}</author>
+    <author>tc={82e76301-cf47-40bb-b34f-dba836074c06}</author>
+    <author>tc={dc8dbba6-e760-4221-ab67-23ddddd4e572}</author>
+    <author>tc={2357850e-c96e-42d7-b5fd-dfce94815ac0}</author>
   </authors>
   <commentList>
-    <comment ref="T2" authorId="0" shapeId="0" xr:uid="{45597FE8-A5BE-4E4C-93E8-EE11830187A8}">
+    <comment ref="T2" authorId="0" shapeId="0" xr:uid="{82E76301-CF47-40BB-B34F-DBA836074C06}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -59,7 +59,7 @@
     https://web.archive.org/web/19990209180306/http://hivdb.stanford.edu/hiv/userguide.asp</t>
       </text>
     </comment>
-    <comment ref="S3" authorId="1" shapeId="0" xr:uid="{5AF53A1D-2122-4BF0-A09A-3FD230718D9D}">
+    <comment ref="S3" authorId="1" shapeId="0" xr:uid="{DC8DBBA6-E760-4221-AB67-23DDDDD4E572}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -67,7 +67,7 @@
     most recent date from their news page https://usidnet.org/2019/03/</t>
       </text>
     </comment>
-    <comment ref="T3" authorId="2" shapeId="0" xr:uid="{E77D8335-66CC-4DB9-ADEA-68353EE4D071}">
+    <comment ref="T3" authorId="2" shapeId="0" xr:uid="{2357850E-C96E-42D7-B5FD-DFCE94815AC0}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -82,10 +82,10 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={8815a28e-f3e7-4c72-b486-fa60101a0d75}</author>
+    <author>tc={c1d7e010-98c0-44a8-83b2-c088c1a491d2}</author>
   </authors>
   <commentList>
-    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{8815A28E-F3E7-4C72-B486-FA60101A0D75}">
+    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{C1D7E010-98C0-44A8-83B2-C088C1A491D2}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="441">
   <si>
     <t>name</t>
   </si>
@@ -590,7 +590,7 @@
     <t>Vela Diagnostics</t>
   </si>
   <si>
-    <t>R2AI171055</t>
+    <t>R24AI171055</t>
   </si>
   <si>
     <t>5U24AI086037</t>
@@ -667,6 +667,9 @@
     <t>citedBy</t>
   </si>
   <si>
+    <t>isRelatedTo</t>
+  </si>
+  <si>
     <t>hasPart</t>
   </si>
   <si>
@@ -812,7 +815,7 @@
     <t>Registry-Supported Publications</t>
   </si>
   <si>
-    <t>https://www.usidnet.net/publications</t>
+    <t>https://usidnet.org/about-the-registry/registry-publications/</t>
   </si>
   <si>
     <t>Disease Matchmaking</t>
@@ -824,6 +827,9 @@
     <t>Custom Dataset Request</t>
   </si>
   <si>
+    <t>https://usidnet.org/registry-data/about-queries/</t>
+  </si>
+  <si>
     <t>Website</t>
   </si>
   <si>
@@ -839,21 +845,21 @@
     <t>https://pubmed.ncbi.nlm.nih.gov/10844935/</t>
   </si>
   <si>
-    <t>V1 Dashboard</t>
-  </si>
-  <si>
-    <t>https://www.usidnet.net/usidnet_v1</t>
-  </si>
-  <si>
-    <t>V2 Dashboard</t>
-  </si>
-  <si>
-    <t>https://www.usidnet.net/usidnet_v2</t>
+    <t>Registry Data Viz</t>
+  </si>
+  <si>
+    <t>https://usidnet.org/registry-data/stats-registry-enrollment/</t>
   </si>
   <si>
     <t>https://rrid.site/data/record/nlx_144509-1/SCR_004672/resolver?q=rrid:scr_004672</t>
   </si>
   <si>
+    <t>USIDNET.net</t>
+  </si>
+  <si>
+    <t>https://usidnet.net</t>
+  </si>
+  <si>
     <t>@type</t>
   </si>
   <si>
@@ -1184,6 +1190,12 @@
     <t>https://www.wikidata.org/wiki/Q30256976</t>
   </si>
   <si>
+    <t>Children's Hospital of Philadelphia</t>
+  </si>
+  <si>
+    <t>CHOP</t>
+  </si>
+  <si>
     <t>prop.description</t>
   </si>
   <si>
@@ -1220,7 +1232,7 @@
     <t>http://purl.obolibrary.org/obo/NCBITaxon_9606</t>
   </si>
   <si>
-    <t>http://edamontology.org/topic_0804</t>
+    <t>http://edamontology.org/topic_3277</t>
   </si>
   <si>
     <t>Patient</t>
@@ -1298,9 +1310,6 @@
     <t>Annotation</t>
   </si>
   <si>
-    <t>Immunology</t>
-  </si>
-  <si>
     <t>sequencing assay</t>
   </si>
   <si>
@@ -1365,6 +1374,9 @@
   </si>
   <si>
     <t>http://edamontology.org/topic_3325</t>
+  </si>
+  <si>
+    <t>Sample Collections</t>
   </si>
   <si>
     <t>inborn error of immunity</t>
@@ -1732,7 +1744,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="G Tsueng" id="{4B15B32C-021F-4F34-A25D-F722ACF38A87}" userId="" providerId="google-sheets"/>
+  <person displayName="G Tsueng" id="{D8B1D967-0729-46FD-BB1D-EAB2E9EE9C1E}" userId="" providerId="google-sheets"/>
 </personList>
 </file>
 
@@ -1934,7 +1946,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="T2" dT="2026-03-17T16:11:12.00" personId="{4B15B32C-021F-4F34-A25D-F722ACF38A87}" id="{45597FE8-A5BE-4E4C-93E8-EE11830187A8}">
+  <threadedComment ref="T2" dT="2026-03-17T16:11:12.00" personId="{D8B1D967-0729-46FD-BB1D-EAB2E9EE9C1E}" id="{82E76301-CF47-40BB-B34F-DBA836074C06}">
     <text>https://web.archive.org/web/19990209180306/http://hivdb.stanford.edu/hiv/userguide.asp</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -1943,7 +1955,7 @@
       </x:ext>
     </extLst>
   </threadedComment>
-  <threadedComment ref="S3" dT="2026-03-17T16:24:57.00" personId="{4B15B32C-021F-4F34-A25D-F722ACF38A87}" id="{5AF53A1D-2122-4BF0-A09A-3FD230718D9D}">
+  <threadedComment ref="S3" dT="2026-03-17T16:24:57.00" personId="{D8B1D967-0729-46FD-BB1D-EAB2E9EE9C1E}" id="{DC8DBBA6-E760-4221-AB67-23DDDDD4E572}">
     <text>most recent date from their news page https://usidnet.org/2019/03/</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -1952,7 +1964,7 @@
       </x:ext>
     </extLst>
   </threadedComment>
-  <threadedComment ref="T3" dT="2026-03-17T16:02:30.00" personId="{4B15B32C-021F-4F34-A25D-F722ACF38A87}" id="{E77D8335-66CC-4DB9-ADEA-68353EE4D071}">
+  <threadedComment ref="T3" dT="2026-03-17T16:02:30.00" personId="{D8B1D967-0729-46FD-BB1D-EAB2E9EE9C1E}" id="{2357850E-C96E-42D7-B5FD-DFCE94815AC0}">
     <text>domain who is registration date</text>
   </threadedComment>
 </ThreadedComments>
@@ -1960,7 +1972,7 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B4" dT="2026-05-21T17:06:50.00" personId="{4B15B32C-021F-4F34-A25D-F722ACF38A87}" id="{8815A28E-F3E7-4C72-B486-FA60101A0D75}">
+  <threadedComment ref="B4" dT="2026-05-21T17:06:50.00" personId="{D8B1D967-0729-46FD-BB1D-EAB2E9EE9C1E}" id="{C1D7E010-98C0-44A8-83B2-C088C1A491D2}">
     <text>from https://hivdb.stanford.edu/cgi-bin/Summary.cgi</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -11094,7 +11106,7 @@
     <col min="1" max="1" width="23.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" ht="13.2">
       <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
@@ -11134,7 +11146,7 @@
         <v>182</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="14.4">
@@ -11142,13 +11154,13 @@
         <v>48</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E3" s="11"/>
     </row>
@@ -11157,16 +11169,16 @@
         <v>48</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>107</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="14.4">
@@ -11174,16 +11186,16 @@
         <v>48</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>107</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="14.4">
@@ -11191,16 +11203,16 @@
         <v>48</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="14.4">
@@ -11208,16 +11220,16 @@
         <v>48</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>107</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="14.4">
@@ -11225,16 +11237,16 @@
         <v>48</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>107</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="14.4">
@@ -11242,16 +11254,16 @@
         <v>48</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>107</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="14.4">
@@ -11259,16 +11271,16 @@
         <v>48</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="14.4">
@@ -11282,10 +11294,10 @@
         <v>107</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="14.4">
@@ -11299,10 +11311,10 @@
         <v>179</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="14.4">
@@ -11316,10 +11328,10 @@
         <v>179</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="14.4">
@@ -11333,10 +11345,10 @@
         <v>179</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="14.4">
@@ -11350,10 +11362,10 @@
         <v>107</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="14.4">
@@ -11367,10 +11379,10 @@
         <v>176</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G16" s="11">
         <v>39339898</v>
@@ -11387,7 +11399,7 @@
         <v>182</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="14.4">
@@ -11395,13 +11407,13 @@
         <v>56</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="14.4">
@@ -11409,16 +11421,16 @@
         <v>56</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>93</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="14.4">
@@ -11426,16 +11438,16 @@
         <v>56</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>93</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="14.4">
@@ -11443,16 +11455,16 @@
         <v>56</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>93</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="14.4">
@@ -11460,16 +11472,16 @@
         <v>56</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="14.4">
@@ -11477,16 +11489,16 @@
         <v>56</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>59</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="14.4">
@@ -11494,16 +11506,16 @@
         <v>56</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="14.4">
@@ -11517,10 +11529,10 @@
         <v>93</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="14.4">
@@ -11534,10 +11546,10 @@
         <v>176</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G26" s="11">
         <v>10844935</v>
@@ -11554,10 +11566,10 @@
         <v>107</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="14.4">
@@ -11565,16 +11577,16 @@
         <v>56</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>238</v>
+        <v>179</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>190</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="14.4">
@@ -11582,17 +11594,21 @@
         <v>56</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>240</v>
-      </c>
+        <v>233</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="14.4">
+      <c r="A30" s="21"/>
+      <c r="B30" s="17"/>
     </row>
     <row r="127" spans="7:8" ht="14.4">
       <c r="G127" s="6"/>
@@ -11727,10 +11743,11 @@
     <hyperlink ref="A27" r:id="rId53" xr:uid="{00000000-0004-0000-0400-000066030000}"/>
     <hyperlink ref="E27" r:id="rId54" xr:uid="{00000000-0004-0000-0400-000067030000}"/>
     <hyperlink ref="A28" r:id="rId55" xr:uid="{00000000-0004-0000-0400-000068030000}"/>
-    <hyperlink ref="E28" r:id="rId56" xr:uid="{00000000-0004-0000-0400-000069030000}"/>
-    <hyperlink ref="A29" r:id="rId57" xr:uid="{00000000-0004-0000-0400-00006A030000}"/>
-    <hyperlink ref="D29" r:id="rId58" xr:uid="{00000000-0004-0000-0400-00006B030000}"/>
-    <hyperlink ref="E29" r:id="rId59" xr:uid="{00000000-0004-0000-0400-00006C030000}"/>
+    <hyperlink ref="D28" r:id="rId56" xr:uid="{00000000-0004-0000-0400-000069030000}"/>
+    <hyperlink ref="E28" r:id="rId57" xr:uid="{00000000-0004-0000-0400-00006A030000}"/>
+    <hyperlink ref="A29" r:id="rId58" xr:uid="{00000000-0004-0000-0400-00006B030000}"/>
+    <hyperlink ref="D29" r:id="rId59" xr:uid="{00000000-0004-0000-0400-00006C030000}"/>
+    <hyperlink ref="E29" r:id="rId60" xr:uid="{00000000-0004-0000-0400-00006D030000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11752,7 +11769,7 @@
         <v>171</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D1" s="11" t="s">
         <v>0</v>
@@ -11761,25 +11778,25 @@
         <v>3</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="G1" s="11" t="s">
         <v>2</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="14.4">
@@ -11787,25 +11804,25 @@
         <v>56</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="14.4">
@@ -11813,25 +11830,25 @@
         <v>56</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G3" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="H3" s="11" t="s">
         <v>256</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="14.4">
@@ -11839,19 +11856,19 @@
         <v>56</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="I4" s="16">
         <v>37889</v>
       </c>
       <c r="K4" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="L4" s="11" t="s">
         <v>261</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -11869,13 +11886,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="21.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" ht="13.2">
       <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
@@ -11886,22 +11903,22 @@
         <v>0</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F1" s="11" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>2</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="14.4">
@@ -11909,25 +11926,25 @@
         <v>48</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="14.4">
@@ -11935,25 +11952,25 @@
         <v>48</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C3" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="G3" s="11" t="s">
         <v>281</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>282</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>283</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>278</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>279</v>
-      </c>
       <c r="H3" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.4">
@@ -11961,25 +11978,25 @@
         <v>48</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="14.4">
@@ -11987,25 +12004,25 @@
         <v>48</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="14.4">
@@ -12013,25 +12030,25 @@
         <v>48</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="14.4">
@@ -12039,22 +12056,22 @@
         <v>48</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="14.4">
@@ -12062,22 +12079,22 @@
         <v>48</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="14.4">
@@ -12085,22 +12102,22 @@
         <v>48</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="14.4">
@@ -12108,22 +12125,22 @@
         <v>48</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="14.4">
@@ -12131,22 +12148,22 @@
         <v>48</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="14.4">
@@ -12154,22 +12171,22 @@
         <v>48</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="14.4">
@@ -12177,22 +12194,22 @@
         <v>48</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E13" s="11" t="s">
+        <v>319</v>
+      </c>
+      <c r="F13" s="11" t="s">
         <v>317</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>315</v>
-      </c>
       <c r="G13" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="14.4">
@@ -12200,22 +12217,22 @@
         <v>48</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="14.4">
@@ -12223,22 +12240,22 @@
         <v>48</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="14.4">
@@ -12246,22 +12263,22 @@
         <v>48</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="14.4">
@@ -12269,22 +12286,22 @@
         <v>48</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="14.4">
@@ -12292,22 +12309,22 @@
         <v>48</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="14.4">
@@ -12315,22 +12332,22 @@
         <v>48</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="14.4">
@@ -12338,22 +12355,22 @@
         <v>48</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="14.4">
@@ -12361,22 +12378,22 @@
         <v>48</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="14.4">
@@ -12384,22 +12401,22 @@
         <v>48</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="14.4">
@@ -12407,22 +12424,22 @@
         <v>48</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="14.4">
@@ -12430,22 +12447,22 @@
         <v>48</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="14.4">
@@ -12453,22 +12470,22 @@
         <v>48</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="14.4">
@@ -12479,13 +12496,27 @@
         <v>131</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>350</v>
+        <v>352</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="14.4">
+      <c r="A27" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>353</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -12517,6 +12548,7 @@
     <hyperlink ref="A25" r:id="rId25" xr:uid="{00000000-0004-0000-0600-000090010000}"/>
     <hyperlink ref="A26" r:id="rId26" xr:uid="{00000000-0004-0000-0600-000091010000}"/>
     <hyperlink ref="H26" r:id="rId27" xr:uid="{00000000-0004-0000-0600-000092010000}"/>
+    <hyperlink ref="A27" r:id="rId28" xr:uid="{00000000-0004-0000-0600-000093010000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12548,7 +12580,7 @@
         <v>172</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.4">
@@ -12556,13 +12588,13 @@
         <v>48</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.4">
@@ -12570,16 +12602,16 @@
         <v>48</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>116</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.4">
@@ -12587,16 +12619,16 @@
         <v>48</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14.4">
@@ -12604,16 +12636,16 @@
         <v>48</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.4">
@@ -12621,13 +12653,13 @@
         <v>48</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.4">
@@ -12635,13 +12667,13 @@
         <v>48</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14.4">
@@ -12649,13 +12681,13 @@
         <v>48</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="14.4">
@@ -12663,13 +12695,13 @@
         <v>48</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14.4">
@@ -12677,13 +12709,13 @@
         <v>48</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="14.4">
@@ -12694,10 +12726,10 @@
         <v>168</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="14.4">
@@ -12705,13 +12737,13 @@
         <v>48</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14.4">
@@ -12719,13 +12751,13 @@
         <v>48</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14.4">
@@ -12733,13 +12765,13 @@
         <v>48</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14.4">
@@ -12747,13 +12779,13 @@
         <v>48</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="14.4">
@@ -12761,13 +12793,13 @@
         <v>48</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14.4">
@@ -12775,13 +12807,13 @@
         <v>48</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="14.4">
@@ -12789,13 +12821,13 @@
         <v>48</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="14.4">
@@ -12803,13 +12835,13 @@
         <v>48</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14.4">
@@ -12817,13 +12849,13 @@
         <v>48</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="14.4">
@@ -12831,13 +12863,13 @@
         <v>48</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="14.4">
@@ -12845,16 +12877,16 @@
         <v>56</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="14.4">
@@ -12862,16 +12894,16 @@
         <v>56</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>131</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="14.4">
@@ -12879,13 +12911,13 @@
         <v>56</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14.4">
@@ -12893,13 +12925,13 @@
         <v>56</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="14.4">
@@ -12907,13 +12939,13 @@
         <v>56</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>389</v>
+        <v>415</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="14.4">
@@ -12921,13 +12953,13 @@
         <v>56</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="14.4">
@@ -12938,10 +12970,10 @@
         <v>168</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="14.4">
@@ -12949,13 +12981,13 @@
         <v>56</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="14.4">
@@ -12963,13 +12995,13 @@
         <v>56</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="14.4">
@@ -12977,13 +13009,13 @@
         <v>56</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="14.4">
@@ -12991,13 +13023,13 @@
         <v>56</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="14.4">
@@ -13005,13 +13037,13 @@
         <v>56</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="14.4">
@@ -13019,13 +13051,13 @@
         <v>56</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="14.4">
@@ -13033,13 +13065,13 @@
         <v>56</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="14.4">
@@ -13047,13 +13079,13 @@
         <v>56</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>
@@ -13150,10 +13182,10 @@
         <v>66</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>18</v>
@@ -13164,13 +13196,13 @@
         <v>48</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="E2" s="16">
         <v>46119</v>
@@ -13181,13 +13213,13 @@
         <v>48</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="E3" s="16">
         <v>46119</v>
@@ -13198,13 +13230,13 @@
         <v>48</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E4" s="16">
         <v>46119</v>

</xml_diff>